<commit_message>
Assegnazioni: pianoforte in aula 17, AIRC in aula 7 secondo orario
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I106"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="48.83203125" customWidth="1"/>
@@ -820,10 +820,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B15" t="str">
-        <v>Teoria gruppo terze (Tromba + Fisarmonica)</v>
+        <v>AIRC · 3B</v>
       </c>
       <c r="C15" t="str">
         <v>temporanea</v>
@@ -832,10 +832,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E15" t="str">
-        <v>13:20</v>
+        <v>10:10</v>
       </c>
       <c r="F15" t="str">
-        <v>14:05</v>
+        <v>11:05</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -849,10 +849,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B16" t="str">
-        <v>Tromba · Musica d'insieme terze</v>
+        <v>AIRC · 3A</v>
       </c>
       <c r="C16" t="str">
         <v>temporanea</v>
@@ -861,10 +861,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E16" t="str">
-        <v>14:05</v>
+        <v>11:05</v>
       </c>
       <c r="F16" t="str">
-        <v>14:50</v>
+        <v>12:10</v>
       </c>
       <c r="G16" t="str">
         <v/>
@@ -878,10 +878,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B17" t="str">
-        <v>Sax · Musica d'insieme terze</v>
+        <v>AIRC · 3C</v>
       </c>
       <c r="C17" t="str">
         <v>temporanea</v>
@@ -890,10 +890,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E17" t="str">
-        <v>14:05</v>
+        <v>12:10</v>
       </c>
       <c r="F17" t="str">
-        <v>14:50</v>
+        <v>13:05</v>
       </c>
       <c r="G17" t="str">
         <v/>
@@ -910,7 +910,7 @@
         <v>7</v>
       </c>
       <c r="B18" t="str">
-        <v>Pianoforte · Musica d'insieme terze</v>
+        <v>AIRC · 1A</v>
       </c>
       <c r="C18" t="str">
         <v>temporanea</v>
@@ -919,10 +919,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E18" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="F18" t="str">
         <v>14:05</v>
-      </c>
-      <c r="F18" t="str">
-        <v>14:50</v>
       </c>
       <c r="G18" t="str">
         <v/>
@@ -936,22 +936,22 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B19" t="str">
-        <v>Fisarmonica · Musica d'insieme terze</v>
+        <v>AIRC · 2A</v>
       </c>
       <c r="C19" t="str">
         <v>temporanea</v>
       </c>
       <c r="D19" t="str">
-        <v>Lunedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E19" t="str">
-        <v>14:05</v>
+        <v>08:05</v>
       </c>
       <c r="F19" t="str">
-        <v>14:50</v>
+        <v>09:05</v>
       </c>
       <c r="G19" t="str">
         <v/>
@@ -965,22 +965,22 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B20" t="str">
-        <v>Tromba · Individuale 1</v>
+        <v>AIRC · 2D</v>
       </c>
       <c r="C20" t="str">
         <v>temporanea</v>
       </c>
       <c r="D20" t="str">
-        <v>Lunedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E20" t="str">
-        <v>14:50</v>
+        <v>10:10</v>
       </c>
       <c r="F20" t="str">
-        <v>15:50</v>
+        <v>11:05</v>
       </c>
       <c r="G20" t="str">
         <v/>
@@ -994,22 +994,22 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B21" t="str">
-        <v>Sax · Individuale 1</v>
+        <v>AIRC · 2B</v>
       </c>
       <c r="C21" t="str">
         <v>temporanea</v>
       </c>
       <c r="D21" t="str">
-        <v>Lunedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E21" t="str">
-        <v>14:50</v>
+        <v>11:05</v>
       </c>
       <c r="F21" t="str">
-        <v>15:50</v>
+        <v>12:10</v>
       </c>
       <c r="G21" t="str">
         <v/>
@@ -1026,19 +1026,19 @@
         <v>7</v>
       </c>
       <c r="B22" t="str">
-        <v>Pianoforte · Individuale 1</v>
+        <v>AIRC · 3D</v>
       </c>
       <c r="C22" t="str">
         <v>temporanea</v>
       </c>
       <c r="D22" t="str">
-        <v>Lunedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E22" t="str">
-        <v>14:50</v>
+        <v>12:10</v>
       </c>
       <c r="F22" t="str">
-        <v>15:50</v>
+        <v>13:05</v>
       </c>
       <c r="G22" t="str">
         <v/>
@@ -1052,22 +1052,22 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B23" t="str">
-        <v>Fisarmonica · Individuale 1</v>
+        <v>AIRC · 1D</v>
       </c>
       <c r="C23" t="str">
         <v>temporanea</v>
       </c>
       <c r="D23" t="str">
-        <v>Lunedì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E23" t="str">
-        <v>14:50</v>
+        <v>10:10</v>
       </c>
       <c r="F23" t="str">
-        <v>15:50</v>
+        <v>11:05</v>
       </c>
       <c r="G23" t="str">
         <v/>
@@ -1081,22 +1081,22 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B24" t="str">
-        <v>Tromba · Individuale 2</v>
+        <v>AIRC · 2C</v>
       </c>
       <c r="C24" t="str">
         <v>temporanea</v>
       </c>
       <c r="D24" t="str">
-        <v>Lunedì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E24" t="str">
-        <v>15:35</v>
+        <v>11:05</v>
       </c>
       <c r="F24" t="str">
-        <v>16:35</v>
+        <v>12:10</v>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -1110,22 +1110,22 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B25" t="str">
-        <v>Sax · Individuale 2</v>
+        <v>AIRC · 1B</v>
       </c>
       <c r="C25" t="str">
         <v>temporanea</v>
       </c>
       <c r="D25" t="str">
-        <v>Lunedì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E25" t="str">
-        <v>15:35</v>
+        <v>12:10</v>
       </c>
       <c r="F25" t="str">
-        <v>16:35</v>
+        <v>13:05</v>
       </c>
       <c r="G25" t="str">
         <v/>
@@ -1142,19 +1142,19 @@
         <v>7</v>
       </c>
       <c r="B26" t="str">
-        <v>Pianoforte · Individuale 2</v>
+        <v>AIRC · 1C</v>
       </c>
       <c r="C26" t="str">
         <v>temporanea</v>
       </c>
       <c r="D26" t="str">
-        <v>Lunedì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E26" t="str">
-        <v>15:35</v>
+        <v>13:05</v>
       </c>
       <c r="F26" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -1168,10 +1168,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27" t="str">
-        <v>Fisarmonica · Individuale 2</v>
+        <v>Teoria gruppo terze (Tromba + Fisarmonica)</v>
       </c>
       <c r="C27" t="str">
         <v>temporanea</v>
@@ -1180,10 +1180,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E27" t="str">
-        <v>15:35</v>
+        <v>13:20</v>
       </c>
       <c r="F27" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G27" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>14</v>
       </c>
       <c r="B28" t="str">
-        <v>Tromba · Individuale 3</v>
+        <v>Tromba · Musica d'insieme terze</v>
       </c>
       <c r="C28" t="str">
         <v>temporanea</v>
@@ -1209,10 +1209,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E28" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F28" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G28" t="str">
         <v/>
@@ -1229,7 +1229,7 @@
         <v>12</v>
       </c>
       <c r="B29" t="str">
-        <v>Sax · Individuale 3</v>
+        <v>Sax · Musica d'insieme terze</v>
       </c>
       <c r="C29" t="str">
         <v>temporanea</v>
@@ -1238,10 +1238,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E29" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F29" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G29" t="str">
         <v/>
@@ -1255,10 +1255,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B30" t="str">
-        <v>Pianoforte · Individuale 3</v>
+        <v>Pianoforte · Musica d'insieme terze</v>
       </c>
       <c r="C30" t="str">
         <v>temporanea</v>
@@ -1267,10 +1267,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E30" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F30" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G30" t="str">
         <v/>
@@ -1287,7 +1287,7 @@
         <v>16</v>
       </c>
       <c r="B31" t="str">
-        <v>Fisarmonica · Individuale 3</v>
+        <v>Fisarmonica · Musica d'insieme terze</v>
       </c>
       <c r="C31" t="str">
         <v>temporanea</v>
@@ -1296,10 +1296,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E31" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F31" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -1313,22 +1313,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B32" t="str">
-        <v>Teoria gruppo seconde (Tromba + Fisarmonica)</v>
+        <v>Tromba · Individuale 1</v>
       </c>
       <c r="C32" t="str">
         <v>temporanea</v>
       </c>
       <c r="D32" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E32" t="str">
-        <v>13:20</v>
+        <v>14:50</v>
       </c>
       <c r="F32" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -1342,22 +1342,22 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B33" t="str">
-        <v>Tromba · Musica d'insieme seconde</v>
+        <v>Sax · Individuale 1</v>
       </c>
       <c r="C33" t="str">
         <v>temporanea</v>
       </c>
       <c r="D33" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E33" t="str">
-        <v>14:05</v>
+        <v>14:50</v>
       </c>
       <c r="F33" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -1371,22 +1371,22 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B34" t="str">
-        <v>Sax · Musica d'insieme seconde</v>
+        <v>Pianoforte · Individuale 1</v>
       </c>
       <c r="C34" t="str">
         <v>temporanea</v>
       </c>
       <c r="D34" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E34" t="str">
-        <v>14:05</v>
+        <v>14:50</v>
       </c>
       <c r="F34" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="G34" t="str">
         <v/>
@@ -1400,22 +1400,22 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B35" t="str">
-        <v>Pianoforte · Musica d'insieme seconde</v>
+        <v>Fisarmonica · Individuale 1</v>
       </c>
       <c r="C35" t="str">
         <v>temporanea</v>
       </c>
       <c r="D35" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E35" t="str">
-        <v>14:05</v>
+        <v>14:50</v>
       </c>
       <c r="F35" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="G35" t="str">
         <v/>
@@ -1429,22 +1429,22 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B36" t="str">
-        <v>Fisarmonica · Musica d'insieme terze</v>
+        <v>Tromba · Individuale 2</v>
       </c>
       <c r="C36" t="str">
         <v>temporanea</v>
       </c>
       <c r="D36" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E36" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="F36" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -1458,22 +1458,22 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B37" t="str">
-        <v>Tromba · Individuale 4</v>
+        <v>Sax · Individuale 2</v>
       </c>
       <c r="C37" t="str">
         <v>temporanea</v>
       </c>
       <c r="D37" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E37" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="F37" t="str">
-        <v>15:50</v>
+        <v>16:20</v>
       </c>
       <c r="G37" t="str">
         <v/>
@@ -1487,22 +1487,22 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B38" t="str">
-        <v>Sax · Individuale 4</v>
+        <v>Pianoforte · Individuale 2</v>
       </c>
       <c r="C38" t="str">
         <v>temporanea</v>
       </c>
       <c r="D38" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E38" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="F38" t="str">
-        <v>15:50</v>
+        <v>16:20</v>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -1516,22 +1516,22 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B39" t="str">
-        <v>Pianoforte · Individuale 4</v>
+        <v>Fisarmonica · Individuale 2</v>
       </c>
       <c r="C39" t="str">
         <v>temporanea</v>
       </c>
       <c r="D39" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E39" t="str">
-        <v>14:50</v>
+        <v>15:35</v>
       </c>
       <c r="F39" t="str">
-        <v>15:50</v>
+        <v>16:20</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -1545,22 +1545,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B40" t="str">
-        <v>Fisarmonica · Individuale 4</v>
+        <v>Tromba · Individuale 3</v>
       </c>
       <c r="C40" t="str">
         <v>temporanea</v>
       </c>
       <c r="D40" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E40" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="F40" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -1574,22 +1574,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B41" t="str">
-        <v>Tromba · Individuale 5</v>
+        <v>Sax · Individuale 3</v>
       </c>
       <c r="C41" t="str">
         <v>temporanea</v>
       </c>
       <c r="D41" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E41" t="str">
-        <v>15:35</v>
+        <v>16:20</v>
       </c>
       <c r="F41" t="str">
-        <v>16:35</v>
+        <v>17:20</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -1603,22 +1603,22 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B42" t="str">
-        <v>Sax · Individuale 5</v>
+        <v>Pianoforte · Individuale 3</v>
       </c>
       <c r="C42" t="str">
         <v>temporanea</v>
       </c>
       <c r="D42" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E42" t="str">
-        <v>15:35</v>
+        <v>16:20</v>
       </c>
       <c r="F42" t="str">
-        <v>16:35</v>
+        <v>17:20</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -1632,22 +1632,22 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B43" t="str">
-        <v>Pianoforte · Individuale 5</v>
+        <v>Fisarmonica · Individuale 3</v>
       </c>
       <c r="C43" t="str">
         <v>temporanea</v>
       </c>
       <c r="D43" t="str">
-        <v>Martedì</v>
+        <v>Lunedì</v>
       </c>
       <c r="E43" t="str">
-        <v>15:35</v>
+        <v>16:20</v>
       </c>
       <c r="F43" t="str">
-        <v>16:35</v>
+        <v>17:20</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -1661,10 +1661,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B44" t="str">
-        <v>Fisarmonica · Individuale 5</v>
+        <v>Teoria gruppo seconde (Tromba + Fisarmonica)</v>
       </c>
       <c r="C44" t="str">
         <v>temporanea</v>
@@ -1673,10 +1673,10 @@
         <v>Martedì</v>
       </c>
       <c r="E44" t="str">
-        <v>15:35</v>
+        <v>13:20</v>
       </c>
       <c r="F44" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G44" t="str">
         <v/>
@@ -1693,7 +1693,7 @@
         <v>14</v>
       </c>
       <c r="B45" t="str">
-        <v>Tromba · Individuale 6</v>
+        <v>Tromba · Musica d'insieme seconde</v>
       </c>
       <c r="C45" t="str">
         <v>temporanea</v>
@@ -1702,10 +1702,10 @@
         <v>Martedì</v>
       </c>
       <c r="E45" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F45" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G45" t="str">
         <v/>
@@ -1722,7 +1722,7 @@
         <v>12</v>
       </c>
       <c r="B46" t="str">
-        <v>Sax · Individuale 6</v>
+        <v>Sax · Musica d'insieme seconde</v>
       </c>
       <c r="C46" t="str">
         <v>temporanea</v>
@@ -1731,10 +1731,10 @@
         <v>Martedì</v>
       </c>
       <c r="E46" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F46" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G46" t="str">
         <v/>
@@ -1748,10 +1748,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B47" t="str">
-        <v>Pianoforte · Individuale 6</v>
+        <v>Pianoforte · Musica d'insieme seconde</v>
       </c>
       <c r="C47" t="str">
         <v>temporanea</v>
@@ -1760,10 +1760,10 @@
         <v>Martedì</v>
       </c>
       <c r="E47" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F47" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G47" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>16</v>
       </c>
       <c r="B48" t="str">
-        <v>Fisarmonica · Individuale 6</v>
+        <v>Fisarmonica · Musica d'insieme terze</v>
       </c>
       <c r="C48" t="str">
         <v>temporanea</v>
@@ -1789,10 +1789,10 @@
         <v>Martedì</v>
       </c>
       <c r="E48" t="str">
-        <v>16:20</v>
+        <v>14:05</v>
       </c>
       <c r="F48" t="str">
-        <v>17:20</v>
+        <v>14:50</v>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -1809,19 +1809,19 @@
         <v>14</v>
       </c>
       <c r="B49" t="str">
-        <v>Tromba · Individuale 7</v>
+        <v>Tromba · Individuale 4</v>
       </c>
       <c r="C49" t="str">
         <v>temporanea</v>
       </c>
       <c r="D49" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E49" t="str">
-        <v>13:20</v>
+        <v>14:50</v>
       </c>
       <c r="F49" t="str">
-        <v>14:20</v>
+        <v>15:35</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -1838,19 +1838,19 @@
         <v>12</v>
       </c>
       <c r="B50" t="str">
-        <v>Sax · Individuale 7</v>
+        <v>Sax · Individuale 4</v>
       </c>
       <c r="C50" t="str">
         <v>temporanea</v>
       </c>
       <c r="D50" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E50" t="str">
-        <v>13:20</v>
+        <v>14:50</v>
       </c>
       <c r="F50" t="str">
-        <v>14:20</v>
+        <v>15:35</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -1864,22 +1864,22 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B51" t="str">
-        <v>Pianoforte · Individuale 7</v>
+        <v>Pianoforte · Individuale 4</v>
       </c>
       <c r="C51" t="str">
         <v>temporanea</v>
       </c>
       <c r="D51" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E51" t="str">
-        <v>13:20</v>
+        <v>14:50</v>
       </c>
       <c r="F51" t="str">
-        <v>14:20</v>
+        <v>15:35</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -1896,19 +1896,19 @@
         <v>16</v>
       </c>
       <c r="B52" t="str">
-        <v>Fisarmonica · Individuale 7</v>
+        <v>Fisarmonica · Individuale 4</v>
       </c>
       <c r="C52" t="str">
         <v>temporanea</v>
       </c>
       <c r="D52" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E52" t="str">
-        <v>13:20</v>
+        <v>14:50</v>
       </c>
       <c r="F52" t="str">
-        <v>14:20</v>
+        <v>15:35</v>
       </c>
       <c r="G52" t="str">
         <v/>
@@ -1925,19 +1925,19 @@
         <v>14</v>
       </c>
       <c r="B53" t="str">
-        <v>Tromba · Individuale 8</v>
+        <v>Tromba · Individuale 5</v>
       </c>
       <c r="C53" t="str">
         <v>temporanea</v>
       </c>
       <c r="D53" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E53" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="F53" t="str">
-        <v>15:05</v>
+        <v>16:20</v>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -1954,19 +1954,19 @@
         <v>12</v>
       </c>
       <c r="B54" t="str">
-        <v>Sax · Individuale 8</v>
+        <v>Sax · Individuale 5</v>
       </c>
       <c r="C54" t="str">
         <v>temporanea</v>
       </c>
       <c r="D54" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E54" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="F54" t="str">
-        <v>15:05</v>
+        <v>16:20</v>
       </c>
       <c r="G54" t="str">
         <v/>
@@ -1980,22 +1980,22 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B55" t="str">
-        <v>Pianoforte · Individuale 8</v>
+        <v>Pianoforte · Individuale 5</v>
       </c>
       <c r="C55" t="str">
         <v>temporanea</v>
       </c>
       <c r="D55" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E55" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="F55" t="str">
-        <v>15:05</v>
+        <v>16:20</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -2012,19 +2012,19 @@
         <v>16</v>
       </c>
       <c r="B56" t="str">
-        <v>Fisarmonica · Individuale 8</v>
+        <v>Fisarmonica · Individuale 5</v>
       </c>
       <c r="C56" t="str">
         <v>temporanea</v>
       </c>
       <c r="D56" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E56" t="str">
-        <v>14:05</v>
+        <v>15:35</v>
       </c>
       <c r="F56" t="str">
-        <v>15:05</v>
+        <v>16:20</v>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -2041,19 +2041,19 @@
         <v>14</v>
       </c>
       <c r="B57" t="str">
-        <v>Tromba · Individuale 9</v>
+        <v>Tromba · Individuale 6</v>
       </c>
       <c r="C57" t="str">
         <v>temporanea</v>
       </c>
       <c r="D57" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E57" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="F57" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G57" t="str">
         <v/>
@@ -2070,19 +2070,19 @@
         <v>12</v>
       </c>
       <c r="B58" t="str">
-        <v>Sax · Individuale 9</v>
+        <v>Sax · Individuale 6</v>
       </c>
       <c r="C58" t="str">
         <v>temporanea</v>
       </c>
       <c r="D58" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E58" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="F58" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G58" t="str">
         <v/>
@@ -2096,22 +2096,22 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B59" t="str">
-        <v>Pianoforte · Individuale 9</v>
+        <v>Pianoforte · Individuale 6</v>
       </c>
       <c r="C59" t="str">
         <v>temporanea</v>
       </c>
       <c r="D59" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E59" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="F59" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G59" t="str">
         <v/>
@@ -2128,19 +2128,19 @@
         <v>16</v>
       </c>
       <c r="B60" t="str">
-        <v>Fisarmonica · Individuale 9</v>
+        <v>Fisarmonica · Individuale 6</v>
       </c>
       <c r="C60" t="str">
         <v>temporanea</v>
       </c>
       <c r="D60" t="str">
-        <v>Mercoledì</v>
+        <v>Martedì</v>
       </c>
       <c r="E60" t="str">
-        <v>14:50</v>
+        <v>16:20</v>
       </c>
       <c r="F60" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G60" t="str">
         <v/>
@@ -2154,10 +2154,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B61" t="str">
-        <v>Sax · Individuale 10</v>
+        <v>Tromba · Individuale 7</v>
       </c>
       <c r="C61" t="str">
         <v>temporanea</v>
@@ -2166,10 +2166,10 @@
         <v>Mercoledì</v>
       </c>
       <c r="E61" t="str">
-        <v>15:35</v>
+        <v>13:20</v>
       </c>
       <c r="F61" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G61" t="str">
         <v/>
@@ -2183,10 +2183,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B62" t="str">
-        <v>Pianoforte · Individuale 10</v>
+        <v>Sax · Individuale 7</v>
       </c>
       <c r="C62" t="str">
         <v>temporanea</v>
@@ -2195,10 +2195,10 @@
         <v>Mercoledì</v>
       </c>
       <c r="E62" t="str">
-        <v>15:35</v>
+        <v>13:20</v>
       </c>
       <c r="F62" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G62" t="str">
         <v/>
@@ -2212,10 +2212,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B63" t="str">
-        <v>Sax · Individuale 13</v>
+        <v>Pianoforte · Individuale 7</v>
       </c>
       <c r="C63" t="str">
         <v>temporanea</v>
@@ -2224,10 +2224,10 @@
         <v>Mercoledì</v>
       </c>
       <c r="E63" t="str">
-        <v>16:20</v>
+        <v>13:20</v>
       </c>
       <c r="F63" t="str">
-        <v>17:20</v>
+        <v>14:05</v>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -2241,10 +2241,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B64" t="str">
-        <v>Pianoforte · Individuale 13</v>
+        <v>Fisarmonica · Individuale 7</v>
       </c>
       <c r="C64" t="str">
         <v>temporanea</v>
@@ -2253,10 +2253,10 @@
         <v>Mercoledì</v>
       </c>
       <c r="E64" t="str">
-        <v>16:20</v>
+        <v>13:20</v>
       </c>
       <c r="F64" t="str">
-        <v>17:20</v>
+        <v>14:05</v>
       </c>
       <c r="G64" t="str">
         <v/>
@@ -2273,19 +2273,19 @@
         <v>14</v>
       </c>
       <c r="B65" t="str">
-        <v>Tromba · Individuale 10 Prime S.L.</v>
+        <v>Tromba · Individuale 8</v>
       </c>
       <c r="C65" t="str">
         <v>temporanea</v>
       </c>
       <c r="D65" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E65" t="str">
-        <v>13:20</v>
+        <v>14:05</v>
       </c>
       <c r="F65" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="G65" t="str">
         <v/>
@@ -2299,22 +2299,22 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B66" t="str">
-        <v>Fisarmonica · Individuale 10 Prime S.L.</v>
+        <v>Sax · Individuale 8</v>
       </c>
       <c r="C66" t="str">
         <v>temporanea</v>
       </c>
       <c r="D66" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E66" t="str">
-        <v>13:20</v>
+        <v>14:05</v>
       </c>
       <c r="F66" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -2328,22 +2328,22 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B67" t="str">
-        <v>Sax · Individuale 11 Prime S.L.</v>
+        <v>Pianoforte · Individuale 8</v>
       </c>
       <c r="C67" t="str">
         <v>temporanea</v>
       </c>
       <c r="D67" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E67" t="str">
-        <v>13:20</v>
+        <v>14:05</v>
       </c>
       <c r="F67" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="G67" t="str">
         <v/>
@@ -2357,22 +2357,22 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B68" t="str">
-        <v>Pianoforte · Individuale 11 Prime S.L.</v>
+        <v>Fisarmonica · Individuale 8</v>
       </c>
       <c r="C68" t="str">
         <v>temporanea</v>
       </c>
       <c r="D68" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E68" t="str">
-        <v>13:20</v>
+        <v>14:05</v>
       </c>
       <c r="F68" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -2389,19 +2389,19 @@
         <v>14</v>
       </c>
       <c r="B69" t="str">
-        <v>Tromba · Musica d'insieme prime</v>
+        <v>Tromba · Individuale 9</v>
       </c>
       <c r="C69" t="str">
         <v>temporanea</v>
       </c>
       <c r="D69" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E69" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="F69" t="str">
-        <v>15:05</v>
+        <v>15:50</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -2418,19 +2418,19 @@
         <v>12</v>
       </c>
       <c r="B70" t="str">
-        <v>Sax · Musica d'insieme prime</v>
+        <v>Sax · Individuale 9</v>
       </c>
       <c r="C70" t="str">
         <v>temporanea</v>
       </c>
       <c r="D70" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E70" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="F70" t="str">
-        <v>15:05</v>
+        <v>15:35</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -2444,22 +2444,22 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B71" t="str">
-        <v>Pianoforte · Musica d'insieme prime</v>
+        <v>Pianoforte · Individuale 9</v>
       </c>
       <c r="C71" t="str">
         <v>temporanea</v>
       </c>
       <c r="D71" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E71" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="F71" t="str">
-        <v>15:05</v>
+        <v>15:35</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -2476,19 +2476,19 @@
         <v>16</v>
       </c>
       <c r="B72" t="str">
-        <v>Fisarmonica · Musica d'insieme prime</v>
+        <v>Fisarmonica · Individuale 9</v>
       </c>
       <c r="C72" t="str">
         <v>temporanea</v>
       </c>
       <c r="D72" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E72" t="str">
-        <v>14:20</v>
+        <v>14:50</v>
       </c>
       <c r="F72" t="str">
-        <v>15:05</v>
+        <v>15:50</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -2502,22 +2502,22 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B73" t="str">
-        <v>Tromba · Individuale 11 (no prime)</v>
+        <v>Sax · Individuale 10</v>
       </c>
       <c r="C73" t="str">
         <v>temporanea</v>
       </c>
       <c r="D73" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E73" t="str">
-        <v>15:05</v>
+        <v>15:35</v>
       </c>
       <c r="F73" t="str">
-        <v>16:05</v>
+        <v>16:20</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -2531,22 +2531,22 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B74" t="str">
-        <v>Pianoforte · Individuale 12 (no prime)</v>
+        <v>Pianoforte · Individuale 10</v>
       </c>
       <c r="C74" t="str">
         <v>temporanea</v>
       </c>
       <c r="D74" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E74" t="str">
-        <v>15:05</v>
+        <v>15:35</v>
       </c>
       <c r="F74" t="str">
-        <v>16:05</v>
+        <v>16:20</v>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -2560,22 +2560,22 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B75" t="str">
-        <v>Teoria gruppo prime (Sax + Fisarmonica)</v>
+        <v>Sax · Individuale 13</v>
       </c>
       <c r="C75" t="str">
         <v>temporanea</v>
       </c>
       <c r="D75" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E75" t="str">
-        <v>15:05</v>
+        <v>16:20</v>
       </c>
       <c r="F75" t="str">
-        <v>15:50</v>
+        <v>17:20</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -2589,22 +2589,22 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B76" t="str">
-        <v>Tromba · Individuale 12</v>
+        <v>Pianoforte · Individuale 13</v>
       </c>
       <c r="C76" t="str">
         <v>temporanea</v>
       </c>
       <c r="D76" t="str">
-        <v>Giovedì</v>
+        <v>Mercoledì</v>
       </c>
       <c r="E76" t="str">
-        <v>15:50</v>
+        <v>16:20</v>
       </c>
       <c r="F76" t="str">
-        <v>16:50</v>
+        <v>17:20</v>
       </c>
       <c r="G76" t="str">
         <v/>
@@ -2618,10 +2618,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B77" t="str">
-        <v>Sax · Individuale 12</v>
+        <v>Tromba · Individuale 10 Prime S.L.</v>
       </c>
       <c r="C77" t="str">
         <v>temporanea</v>
@@ -2630,10 +2630,10 @@
         <v>Giovedì</v>
       </c>
       <c r="E77" t="str">
-        <v>15:50</v>
+        <v>13:20</v>
       </c>
       <c r="F77" t="str">
-        <v>16:50</v>
+        <v>14:20</v>
       </c>
       <c r="G77" t="str">
         <v/>
@@ -2647,10 +2647,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B78" t="str">
-        <v>Pianoforte · Individuale 13</v>
+        <v>Fisarmonica · Individuale 10 Prime S.L.</v>
       </c>
       <c r="C78" t="str">
         <v>temporanea</v>
@@ -2659,10 +2659,10 @@
         <v>Giovedì</v>
       </c>
       <c r="E78" t="str">
-        <v>15:50</v>
+        <v>13:20</v>
       </c>
       <c r="F78" t="str">
-        <v>16:50</v>
+        <v>14:20</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -2676,10 +2676,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B79" t="str">
-        <v>Fisarmonica · Individuale 11</v>
+        <v>Sax · Individuale 11 Prime S.L.</v>
       </c>
       <c r="C79" t="str">
         <v>temporanea</v>
@@ -2688,10 +2688,10 @@
         <v>Giovedì</v>
       </c>
       <c r="E79" t="str">
-        <v>15:50</v>
+        <v>13:20</v>
       </c>
       <c r="F79" t="str">
-        <v>16:50</v>
+        <v>14:20</v>
       </c>
       <c r="G79" t="str">
         <v/>
@@ -2705,10 +2705,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B80" t="str">
-        <v>Fisarmonica · Individuale 12</v>
+        <v>Pianoforte · Individuale 11 Prime S.L.</v>
       </c>
       <c r="C80" t="str">
         <v>temporanea</v>
@@ -2717,10 +2717,10 @@
         <v>Giovedì</v>
       </c>
       <c r="E80" t="str">
-        <v>16:35</v>
+        <v>13:20</v>
       </c>
       <c r="F80" t="str">
-        <v>17:35</v>
+        <v>14:20</v>
       </c>
       <c r="G80" t="str">
         <v/>
@@ -2737,19 +2737,19 @@
         <v>14</v>
       </c>
       <c r="B81" t="str">
-        <v>Tromba · Individuale 13</v>
+        <v>Tromba · Musica d'insieme prime</v>
       </c>
       <c r="C81" t="str">
         <v>temporanea</v>
       </c>
       <c r="D81" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E81" t="str">
-        <v>13:20</v>
+        <v>14:20</v>
       </c>
       <c r="F81" t="str">
-        <v>14:20</v>
+        <v>15:05</v>
       </c>
       <c r="G81" t="str">
         <v/>
@@ -2763,19 +2763,19 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B82" t="str">
-        <v>Tromba · Individuale 14</v>
+        <v>Sax · Musica d'insieme prime</v>
       </c>
       <c r="C82" t="str">
         <v>temporanea</v>
       </c>
       <c r="D82" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E82" t="str">
-        <v>14:05</v>
+        <v>14:20</v>
       </c>
       <c r="F82" t="str">
         <v>15:05</v>
@@ -2792,22 +2792,22 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B83" t="str">
-        <v>Tromba · Individuale 15</v>
+        <v>Pianoforte · Musica d'insieme prime</v>
       </c>
       <c r="C83" t="str">
         <v>temporanea</v>
       </c>
       <c r="D83" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E83" t="str">
-        <v>14:50</v>
+        <v>14:20</v>
       </c>
       <c r="F83" t="str">
-        <v>15:50</v>
+        <v>15:05</v>
       </c>
       <c r="G83" t="str">
         <v/>
@@ -2821,22 +2821,22 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B84" t="str">
-        <v>Tromba · Individuale 16</v>
+        <v>Fisarmonica · Musica d'insieme prime</v>
       </c>
       <c r="C84" t="str">
         <v>temporanea</v>
       </c>
       <c r="D84" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E84" t="str">
-        <v>15:35</v>
+        <v>14:20</v>
       </c>
       <c r="F84" t="str">
-        <v>16:35</v>
+        <v>15:05</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -2850,22 +2850,22 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B85" t="str">
-        <v>Sax · Individuale 14</v>
+        <v>Tromba · Individuale 11 (no prime)</v>
       </c>
       <c r="C85" t="str">
         <v>temporanea</v>
       </c>
       <c r="D85" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E85" t="str">
-        <v>13:20</v>
+        <v>15:05</v>
       </c>
       <c r="F85" t="str">
-        <v>14:20</v>
+        <v>15:50</v>
       </c>
       <c r="G85" t="str">
         <v/>
@@ -2879,22 +2879,22 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B86" t="str">
-        <v>Sax · Individuale 15</v>
+        <v>Pianoforte · Individuale 12 (no prime)</v>
       </c>
       <c r="C86" t="str">
         <v>temporanea</v>
       </c>
       <c r="D86" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E86" t="str">
-        <v>14:05</v>
+        <v>15:05</v>
       </c>
       <c r="F86" t="str">
-        <v>15:05</v>
+        <v>15:50</v>
       </c>
       <c r="G86" t="str">
         <v/>
@@ -2911,16 +2911,16 @@
         <v>12</v>
       </c>
       <c r="B87" t="str">
-        <v>Sax · Individuale 16</v>
+        <v>Teoria gruppo prime (Sax + Fisarmonica)</v>
       </c>
       <c r="C87" t="str">
         <v>temporanea</v>
       </c>
       <c r="D87" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E87" t="str">
-        <v>14:50</v>
+        <v>15:05</v>
       </c>
       <c r="F87" t="str">
         <v>15:50</v>
@@ -2937,22 +2937,22 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B88" t="str">
-        <v>Sax · Individuale 17</v>
+        <v>Tromba · Individuale 12</v>
       </c>
       <c r="C88" t="str">
         <v>temporanea</v>
       </c>
       <c r="D88" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E88" t="str">
-        <v>15:35</v>
+        <v>15:50</v>
       </c>
       <c r="F88" t="str">
-        <v>16:35</v>
+        <v>16:50</v>
       </c>
       <c r="G88" t="str">
         <v/>
@@ -2969,19 +2969,19 @@
         <v>12</v>
       </c>
       <c r="B89" t="str">
-        <v>Sax · Individuale 18</v>
+        <v>Sax · Individuale 12</v>
       </c>
       <c r="C89" t="str">
         <v>temporanea</v>
       </c>
       <c r="D89" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E89" t="str">
-        <v>16:20</v>
+        <v>15:50</v>
       </c>
       <c r="F89" t="str">
-        <v>17:20</v>
+        <v>16:50</v>
       </c>
       <c r="G89" t="str">
         <v/>
@@ -2995,22 +2995,22 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B90" t="str">
-        <v>Pianoforte · Individuale 15</v>
+        <v>Pianoforte · Individuale 13</v>
       </c>
       <c r="C90" t="str">
         <v>temporanea</v>
       </c>
       <c r="D90" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E90" t="str">
-        <v>13:20</v>
+        <v>15:50</v>
       </c>
       <c r="F90" t="str">
-        <v>14:20</v>
+        <v>16:50</v>
       </c>
       <c r="G90" t="str">
         <v/>
@@ -3024,22 +3024,22 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B91" t="str">
-        <v>Pianoforte · Individuale 16</v>
+        <v>Fisarmonica · Individuale 11</v>
       </c>
       <c r="C91" t="str">
         <v>temporanea</v>
       </c>
       <c r="D91" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E91" t="str">
-        <v>14:05</v>
+        <v>15:50</v>
       </c>
       <c r="F91" t="str">
-        <v>15:05</v>
+        <v>16:35</v>
       </c>
       <c r="G91" t="str">
         <v/>
@@ -3053,22 +3053,22 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B92" t="str">
-        <v>Pianoforte · Individuale 17</v>
+        <v>Fisarmonica · Individuale 12</v>
       </c>
       <c r="C92" t="str">
         <v>temporanea</v>
       </c>
       <c r="D92" t="str">
-        <v>Venerdì</v>
+        <v>Giovedì</v>
       </c>
       <c r="E92" t="str">
-        <v>14:50</v>
+        <v>16:35</v>
       </c>
       <c r="F92" t="str">
-        <v>15:50</v>
+        <v>17:35</v>
       </c>
       <c r="G92" t="str">
         <v/>
@@ -3082,10 +3082,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B93" t="str">
-        <v>Pianoforte · Individuale 18</v>
+        <v>Tromba · Individuale 13</v>
       </c>
       <c r="C93" t="str">
         <v>temporanea</v>
@@ -3094,10 +3094,10 @@
         <v>Venerdì</v>
       </c>
       <c r="E93" t="str">
-        <v>15:35</v>
+        <v>13:20</v>
       </c>
       <c r="F93" t="str">
-        <v>16:35</v>
+        <v>14:05</v>
       </c>
       <c r="G93" t="str">
         <v/>
@@ -3111,10 +3111,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B94" t="str">
-        <v>Pianoforte · Individuale 19</v>
+        <v>Tromba · Individuale 14</v>
       </c>
       <c r="C94" t="str">
         <v>temporanea</v>
@@ -3123,24 +3123,372 @@
         <v>Venerdì</v>
       </c>
       <c r="E94" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="F94" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="G94" t="str">
+        <v/>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>14</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Tromba · Individuale 15</v>
+      </c>
+      <c r="C95" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E95" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="F95" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>14</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Tromba · Individuale 16</v>
+      </c>
+      <c r="C96" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E96" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="F96" t="str">
+        <v>16:35</v>
+      </c>
+      <c r="G96" t="str">
+        <v/>
+      </c>
+      <c r="H96" t="str">
+        <v/>
+      </c>
+      <c r="I96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>12</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Sax · Individuale 14</v>
+      </c>
+      <c r="C97" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E97" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="F97" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="G97" t="str">
+        <v/>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>12</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Sax · Individuale 15</v>
+      </c>
+      <c r="C98" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E98" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="F98" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="G98" t="str">
+        <v/>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>12</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Sax · Individuale 16</v>
+      </c>
+      <c r="C99" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E99" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="F99" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="G99" t="str">
+        <v/>
+      </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>12</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Sax · Individuale 17</v>
+      </c>
+      <c r="C100" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E100" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="F100" t="str">
         <v>16:20</v>
       </c>
-      <c r="F94" t="str">
+      <c r="G100" t="str">
+        <v/>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>12</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Sax · Individuale 18</v>
+      </c>
+      <c r="C101" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E101" t="str">
+        <v>16:20</v>
+      </c>
+      <c r="F101" t="str">
         <v>17:20</v>
       </c>
-      <c r="G94" t="str">
-        <v/>
-      </c>
-      <c r="H94" t="str">
-        <v/>
-      </c>
-      <c r="I94" t="str">
+      <c r="G101" t="str">
+        <v/>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>17</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Pianoforte · Individuale 15</v>
+      </c>
+      <c r="C102" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E102" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="F102" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="G102" t="str">
+        <v/>
+      </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>17</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Pianoforte · Individuale 16</v>
+      </c>
+      <c r="C103" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E103" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="F103" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="G103" t="str">
+        <v/>
+      </c>
+      <c r="H103" t="str">
+        <v/>
+      </c>
+      <c r="I103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>17</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Pianoforte · Individuale 17</v>
+      </c>
+      <c r="C104" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E104" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="F104" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="G104" t="str">
+        <v/>
+      </c>
+      <c r="H104" t="str">
+        <v/>
+      </c>
+      <c r="I104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>17</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Pianoforte · Individuale 18</v>
+      </c>
+      <c r="C105" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E105" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="F105" t="str">
+        <v>16:20</v>
+      </c>
+      <c r="G105" t="str">
+        <v/>
+      </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+      <c r="I105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>17</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Pianoforte · Individuale 19</v>
+      </c>
+      <c r="C106" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E106" t="str">
+        <v>16:20</v>
+      </c>
+      <c r="F106" t="str">
+        <v>17:20</v>
+      </c>
+      <c r="G106" t="str">
+        <v/>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I106"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Assegnazioni: francese e spagnolo (2ª lingua) dall'orario
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I126"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="48.83203125" customWidth="1"/>
@@ -3486,9 +3486,589 @@
         <v/>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>12</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Francese · 3A-3C</v>
+      </c>
+      <c r="C107" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E107" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F107" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="G107" t="str">
+        <v/>
+      </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+      <c r="I107" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>19</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Spagnolo · 3A-3C</v>
+      </c>
+      <c r="C108" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E108" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F108" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="G108" t="str">
+        <v/>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>12</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Francese · 1B-1D</v>
+      </c>
+      <c r="C109" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E109" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="F109" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="G109" t="str">
+        <v/>
+      </c>
+      <c r="H109" t="str">
+        <v/>
+      </c>
+      <c r="I109" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>19</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Spagnolo · 1B-1D</v>
+      </c>
+      <c r="C110" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E110" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="F110" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>12</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Francese · 1A-1C</v>
+      </c>
+      <c r="C111" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E111" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F111" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="G111" t="str">
+        <v/>
+      </c>
+      <c r="H111" t="str">
+        <v/>
+      </c>
+      <c r="I111" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>19</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Spagnolo · 1A-1C</v>
+      </c>
+      <c r="C112" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Mercoledì</v>
+      </c>
+      <c r="E112" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F112" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="G112" t="str">
+        <v/>
+      </c>
+      <c r="H112" t="str">
+        <v/>
+      </c>
+      <c r="I112" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>12</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Francese · 1B-1D</v>
+      </c>
+      <c r="C113" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E113" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F113" t="str">
+        <v>09:05</v>
+      </c>
+      <c r="G113" t="str">
+        <v/>
+      </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>19</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Spagnolo · 1B-1D</v>
+      </c>
+      <c r="C114" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E114" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F114" t="str">
+        <v>09:05</v>
+      </c>
+      <c r="G114" t="str">
+        <v/>
+      </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>12</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Francese · 1A-1C</v>
+      </c>
+      <c r="C115" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E115" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="F115" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="G115" t="str">
+        <v/>
+      </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>19</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Spagnolo · 1A-1C</v>
+      </c>
+      <c r="C116" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E116" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="F116" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="G116" t="str">
+        <v/>
+      </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>12</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Francese · 2B-2D</v>
+      </c>
+      <c r="C117" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E117" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F117" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="G117" t="str">
+        <v/>
+      </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>19</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Spagnolo · 2B-2D</v>
+      </c>
+      <c r="C118" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E118" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F118" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="G118" t="str">
+        <v/>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>12</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Francese · 2A-2C</v>
+      </c>
+      <c r="C119" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E119" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="F119" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="G119" t="str">
+        <v/>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>19</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Spagnolo · 2A-2C</v>
+      </c>
+      <c r="C120" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Giovedì</v>
+      </c>
+      <c r="E120" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="F120" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="G120" t="str">
+        <v/>
+      </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>12</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Francese · 3B-3D</v>
+      </c>
+      <c r="C121" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E121" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F121" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="G121" t="str">
+        <v/>
+      </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>19</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Spagnolo · 3B-3D</v>
+      </c>
+      <c r="C122" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E122" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="F122" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="G122" t="str">
+        <v/>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>12</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Francese · 2A-2C</v>
+      </c>
+      <c r="C123" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E123" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F123" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="G123" t="str">
+        <v/>
+      </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>19</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Spagnolo · 2A-2C</v>
+      </c>
+      <c r="C124" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E124" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="F124" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="G124" t="str">
+        <v/>
+      </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>12</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Francese · 2B-2D</v>
+      </c>
+      <c r="C125" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E125" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="F125" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="G125" t="str">
+        <v/>
+      </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v>Basso R.</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>19</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Spagnolo · 2B-2D</v>
+      </c>
+      <c r="C126" t="str">
+        <v>temporanea</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Venerdì</v>
+      </c>
+      <c r="E126" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="F126" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="G126" t="str">
+        <v/>
+      </c>
+      <c r="H126" t="str">
+        <v/>
+      </c>
+      <c r="I126" t="str">
+        <v>Martinelli</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I106"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I126"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Laboratori di orientamento: aula 1, 8:30-13:00
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -7730,8 +7730,8 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="str">
-        <v/>
+      <c r="A210">
+        <v>1</v>
       </c>
       <c r="B210" t="str">
         <v>Orientamento: laboratori scuole secondarie (classi 3)</v>
@@ -7743,10 +7743,10 @@
         <v>Lunedì</v>
       </c>
       <c r="E210" t="str">
-        <v>08:05</v>
+        <v>08:30</v>
       </c>
       <c r="F210" t="str">
-        <v>13:05</v>
+        <v>13:00</v>
       </c>
       <c r="G210" t="str">
         <v>2026-11-23</v>
@@ -7758,10 +7758,10 @@
         <v/>
       </c>
       <c r="J210" t="str">
-        <v>Auditorium</v>
+        <v/>
       </c>
       <c r="K210" t="str">
-        <v>terra</v>
+        <v/>
       </c>
     </row>
     <row r="211">
@@ -7870,8 +7870,8 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="str">
-        <v/>
+      <c r="A214">
+        <v>1</v>
       </c>
       <c r="B214" t="str">
         <v>Orientamento: laboratori scuole secondarie (classi 3)</v>
@@ -7883,10 +7883,10 @@
         <v>Venerdì</v>
       </c>
       <c r="E214" t="str">
-        <v>08:05</v>
+        <v>08:30</v>
       </c>
       <c r="F214" t="str">
-        <v>13:05</v>
+        <v>13:00</v>
       </c>
       <c r="G214" t="str">
         <v>2026-11-27</v>
@@ -7898,10 +7898,10 @@
         <v/>
       </c>
       <c r="J214" t="str">
-        <v>Auditorium</v>
+        <v/>
       </c>
       <c r="K214" t="str">
-        <v>terra</v>
+        <v/>
       </c>
     </row>
     <row r="215">
@@ -8010,8 +8010,8 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="str">
-        <v/>
+      <c r="A218">
+        <v>1</v>
       </c>
       <c r="B218" t="str">
         <v>Orientamento: laboratori scuole secondarie (classi 3)</v>
@@ -8023,10 +8023,10 @@
         <v>Martedì</v>
       </c>
       <c r="E218" t="str">
-        <v>08:05</v>
+        <v>08:30</v>
       </c>
       <c r="F218" t="str">
-        <v>13:05</v>
+        <v>13:00</v>
       </c>
       <c r="G218" t="str">
         <v>2026-11-24</v>
@@ -8038,15 +8038,15 @@
         <v/>
       </c>
       <c r="J218" t="str">
-        <v>Auditorium</v>
+        <v/>
       </c>
       <c r="K218" t="str">
-        <v>terra</v>
+        <v/>
       </c>
     </row>
     <row r="219">
-      <c r="A219" t="str">
-        <v/>
+      <c r="A219">
+        <v>1</v>
       </c>
       <c r="B219" t="str">
         <v>Orientamento: laboratori scuole secondarie (classi 3)</v>
@@ -8058,10 +8058,10 @@
         <v>Mercoledì</v>
       </c>
       <c r="E219" t="str">
-        <v>08:05</v>
+        <v>08:30</v>
       </c>
       <c r="F219" t="str">
-        <v>13:05</v>
+        <v>13:00</v>
       </c>
       <c r="G219" t="str">
         <v>2026-11-25</v>
@@ -8073,10 +8073,10 @@
         <v/>
       </c>
       <c r="J219" t="str">
-        <v>Auditorium</v>
+        <v/>
       </c>
       <c r="K219" t="str">
-        <v>terra</v>
+        <v/>
       </c>
     </row>
     <row r="220">

</xml_diff>

<commit_message>
AIRC in aule 12 (lun), 14 (mer, gio); L2 in aula 7
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -906,7 +906,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B15" t="str">
         <v>AIRC · 3B</v>
@@ -941,7 +941,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B16" t="str">
         <v>AIRC · 3A</v>
@@ -976,7 +976,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B17" t="str">
         <v>AIRC · 3C</v>
@@ -1011,7 +1011,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B18" t="str">
         <v>AIRC · 1A</v>
@@ -1046,7 +1046,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B19" t="str">
         <v>AIRC · 2A</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B20" t="str">
         <v>AIRC · 2D</v>
@@ -1116,7 +1116,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B21" t="str">
         <v>AIRC · 2B</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B22" t="str">
         <v>AIRC · 3D</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B23" t="str">
         <v>AIRC · 1D</v>
@@ -1221,7 +1221,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B24" t="str">
         <v>AIRC · 2C</v>
@@ -1256,7 +1256,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B25" t="str">
         <v>AIRC · 1B</v>
@@ -4826,7 +4826,7 @@
     </row>
     <row r="127">
       <c r="A127">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B127" t="str">
         <v>Italiano L2 · Gruppo C (1C, 1D)</v>
@@ -4861,7 +4861,7 @@
     </row>
     <row r="128">
       <c r="A128">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B128" t="str">
         <v>Italiano L2 · Gruppo F (3C)</v>
@@ -4896,7 +4896,7 @@
     </row>
     <row r="129">
       <c r="A129">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B129" t="str">
         <v>Italiano L2 · Gruppo A (1B, 1D, 2A, 2D)</v>
@@ -4931,7 +4931,7 @@
     </row>
     <row r="130">
       <c r="A130">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B130" t="str">
         <v>Italiano L2 · Gruppo A (1B, 1D, 2A, 2D)</v>
@@ -4966,7 +4966,7 @@
     </row>
     <row r="131">
       <c r="A131">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B131" t="str">
         <v>Italiano L2 · Gruppo D (2B, 2C, 2D)</v>
@@ -5001,7 +5001,7 @@
     </row>
     <row r="132">
       <c r="A132">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B132" t="str">
         <v>Italiano L2 · Gruppo B (1A, 1B)</v>
@@ -5036,7 +5036,7 @@
     </row>
     <row r="133">
       <c r="A133">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B133" t="str">
         <v>Italiano L2 · Gruppo E (3A, 3B)</v>
@@ -5071,7 +5071,7 @@
     </row>
     <row r="134">
       <c r="A134">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B134" t="str">
         <v>Italiano L2 · Gruppo C (1C, 1D)</v>
@@ -5106,7 +5106,7 @@
     </row>
     <row r="135">
       <c r="A135">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B135" t="str">
         <v>Italiano L2 · Gruppo B (1A, 1B)</v>
@@ -5141,7 +5141,7 @@
     </row>
     <row r="136">
       <c r="A136">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B136" t="str">
         <v>Italiano L2 · Gruppo F (3C)</v>
@@ -5176,7 +5176,7 @@
     </row>
     <row r="137">
       <c r="A137">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B137" t="str">
         <v>Italiano L2 · Gruppo E (3A, 3B)</v>
@@ -5211,7 +5211,7 @@
     </row>
     <row r="138">
       <c r="A138">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B138" t="str">
         <v>Italiano L2 · Gruppo D (2B, 2C, 2D)</v>

</xml_diff>

<commit_message>
AIRC: lun aula 12, mer aula 14, gio aula 7; L2 aula 7
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -1186,7 +1186,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B23" t="str">
         <v>AIRC · 1D</v>
@@ -1221,7 +1221,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B24" t="str">
         <v>AIRC · 2C</v>
@@ -1256,7 +1256,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B25" t="str">
         <v>AIRC · 1B</v>

</xml_diff>

<commit_message>
AIRC 1C in aula 7
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8YKoioKA4JxzQFPk2TT87
</commit_message>
<xml_diff>
--- a/data/modello-assegnazioni-compilato.xlsx
+++ b/data/modello-assegnazioni-compilato.xlsx
@@ -1157,7 +1157,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -23665,7 +23665,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -23750,7 +23749,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>